<commit_message>
Renombra _rec_tercil a _cat y VARS_REC_TERCIL a VARS_MODELO
Refactor puro, sin cambio de comportamiento, previo a resolver D2. Las
variables dejan de llamarse terciles porque están a punto de dejar de
serlo, y VARS_REC_TERCIL era doblemente engañoso: contenía perper_delito
y comper_gasto, que no son terciles, y "REC" es vocabulario anterior a la
nomenclatura de §4.0.

Se hace antes del cambio de cortes y no después para que cada diff
muestre una sola cosa. Verificado: las seis distribuciones son idénticas
a las de antes del rename y el N del MCA sigue en 49.503.

Incluye el archivado de la página con terciles en
docs/archivo/2025-08-terciles/, con una banda en cada una de las siete
páginas que indica que es una versión congelada y enlaza a la vigente.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/tables/2025/metadata_variables.xlsx
+++ b/output/tables/2025/metadata_variables.xlsx
@@ -1280,7 +1280,7 @@
     <t xml:space="preserve">Fuente: categorizada</t>
   </si>
   <si>
-    <t xml:space="preserve">emper_ep_pct_rec_tercil</t>
+    <t xml:space="preserve">emper_ep_pct_cat</t>
   </si>
   <si>
     <t xml:space="preserve">Inseguridad en Espacio público (tercile)</t>
@@ -1292,7 +1292,7 @@
     <t xml:space="preserve">Entra al modelo (MCA)</t>
   </si>
   <si>
-    <t xml:space="preserve">emper_barrio_pct_rec_tercil</t>
+    <t xml:space="preserve">emper_barrio_pct_cat</t>
   </si>
   <si>
     <t xml:space="preserve">Inseguridad en Barrio (tercile)</t>
@@ -1301,7 +1301,7 @@
     <t xml:space="preserve">1 = Baja inseguridad en el barrio; 2 = Media inseguridad en el barrio; 3 = Alta inseguridad en el barrio; 85 = No aplica; 88 = No sabe; 99 = No responde</t>
   </si>
   <si>
-    <t xml:space="preserve">emper_casa_pct_rec_tercil</t>
+    <t xml:space="preserve">emper_casa_pct_cat</t>
   </si>
   <si>
     <t xml:space="preserve">Inseguridad en Casa (tercile)</t>
@@ -1319,7 +1319,7 @@
     <t xml:space="preserve">perper_p_expos_delito, perper_p_delito_pronostico_1, perper_p_delito_pronostico_2, perper_p_delito_pronostico_3, perper_p_delito_pronostico_4, perper_p_delito_pronostico_6, perper_p_delito_pronostico_9, perper_p_delito_pronostico_10, perper_p_delito_pronostico_11, perper_p_delito_pronostico_5, perper_p_delito_pronostico_7, perper_p_delito_pronostico_8, perper_p_expos_delito, perper_p_delito_pronostico_77, perper_p_delito_pronostico_88, perper_p_delito_pronostico_99</t>
   </si>
   <si>
-    <t xml:space="preserve">comper_pct_rec_tercil</t>
+    <t xml:space="preserve">comper_pct_cat</t>
   </si>
   <si>
     <t xml:space="preserve">Modifica comportamiento (tercile)</t>
@@ -1334,7 +1334,7 @@
     <t xml:space="preserve">0 = No gasta en medidas de seguridad; 1 = Gasta en medidas de seguridad; 88 = No sabe; 99 = No responde</t>
   </si>
   <si>
-    <t xml:space="preserve">comgen_per_pct_rec_tercil</t>
+    <t xml:space="preserve">comgen_per_pct_cat</t>
   </si>
   <si>
     <t xml:space="preserve">Dispone de medidas de seguridad (personales) (tercile)</t>
@@ -1343,7 +1343,7 @@
     <t xml:space="preserve">1 = Baja disposición de medidas vivienda; 2 = Media disposición de medidas vivienda; 3 = Alta disposición de medidas vivienda; 85 = No aplica; 88 = No sabe; 99 = No responde</t>
   </si>
   <si>
-    <t xml:space="preserve">comgen_com_pct_rec_tercil</t>
+    <t xml:space="preserve">comgen_com_pct_cat</t>
   </si>
   <si>
     <t xml:space="preserve">Disponen de medidas de seguridad (comunitarias) (tercile)</t>
@@ -1364,7 +1364,7 @@
     <t xml:space="preserve">C1; C2; C3; C4</t>
   </si>
   <si>
-    <t xml:space="preserve">emper_ep_pct_rec_tercil, emper_barrio_pct_rec_tercil, emper_casa_pct_rec_tercil, perper_delito, comper_pct_rec_tercil, comper_gasto, comgen_per_pct_rec_tercil, comgen_com_pct_rec_tercil</t>
+    <t xml:space="preserve">emper_ep_pct_cat, emper_barrio_pct_cat, emper_casa_pct_cat, perper_delito, comper_pct_cat, comper_gasto, comgen_per_pct_cat, comgen_com_pct_cat</t>
   </si>
   <si>
     <t xml:space="preserve">Resultado del modelo</t>

</xml_diff>